<commit_message>
PFOA blood flows were adjusted to give matching liver and kidney flows but reducing cardiac output by GFR. which is treated as a "lost" flow in the Loccisano et al. model.
</commit_message>
<xml_diff>
--- a/Inputs/PFOA_template_parameters_Model.xlsx
+++ b/Inputs/PFOA_template_parameters_Model.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa.sharepoint.com/sites/ORD/pkwg/Shared Documents/PFAS/PFAS inhalation/pfas_inhalation_pbpk/Inputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="97" documentId="13_ncr:1_{C7746A5F-920D-41F0-A536-A594C5CF14B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0835F917-0AD2-4EE2-B689-A706E57128C5}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="13_ncr:1_{C7746A5F-920D-41F0-A536-A594C5CF14B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89DA856E-E59D-4561-8B3E-D8CC408A3D95}"/>
   <bookViews>
-    <workbookView xWindow="2265" yWindow="345" windowWidth="21600" windowHeight="11100" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="1830" yWindow="1890" windowWidth="21600" windowHeight="12585" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="MaleRat" sheetId="9" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="307" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="240">
   <si>
     <t>Code</t>
   </si>
@@ -744,6 +744,15 @@
   </si>
   <si>
     <t>num.blood.comp</t>
+  </si>
+  <si>
+    <t>Total</t>
+  </si>
+  <si>
+    <t>plasma</t>
+  </si>
+  <si>
+    <t>Fractions of total plasma flow</t>
   </si>
 </sst>
 </file>
@@ -759,7 +768,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -769,6 +778,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -785,7 +800,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -793,6 +808,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -869,10 +885,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1172,7 +1184,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3ADCAA70-43B6-4F02-AE2A-67A6EACE5958}">
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
@@ -1416,7 +1428,7 @@
       </c>
       <c r="E15">
         <f>1-SUM(E76:E85)</f>
-        <v>7.0500000000000118E-2</v>
+        <v>0</v>
       </c>
       <c r="F15" t="s">
         <v>217</v>
@@ -1437,7 +1449,7 @@
         <v>0.84000000000000008</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>0</v>
       </c>
@@ -1457,7 +1469,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>71</v>
       </c>
@@ -1474,7 +1486,7 @@
         <v>414.07</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>27</v>
       </c>
@@ -1488,7 +1500,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
@@ -1502,7 +1514,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>228</v>
       </c>
@@ -1520,7 +1532,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -1534,7 +1546,7 @@
         <v>-0.25</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
@@ -1547,26 +1559,36 @@
       <c r="D24">
         <v>0</v>
       </c>
-      <c r="E24">
+      <c r="E24" s="5">
+        <f>F25*(1-E52)</f>
+        <v>7.0270200000000003</v>
+      </c>
+      <c r="F24" s="5">
+        <v>14</v>
+      </c>
+      <c r="G24" s="5" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="B25" t="s">
+        <v>44</v>
+      </c>
+      <c r="D25">
+        <v>0</v>
+      </c>
+      <c r="F25" s="5">
         <f>F24*(1-E99)</f>
         <v>7.5600000000000005</v>
       </c>
-      <c r="F24">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="B25" t="s">
-        <v>44</v>
-      </c>
-      <c r="D25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G25" s="5" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>142</v>
       </c>
@@ -1583,7 +1605,7 @@
         <v>270000</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>143</v>
       </c>
@@ -1600,7 +1622,7 @@
         <v>67000</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>48</v>
       </c>
@@ -1618,7 +1640,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>144</v>
       </c>
@@ -1635,7 +1657,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>145</v>
       </c>
@@ -1649,7 +1671,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>146</v>
       </c>
@@ -1666,7 +1688,7 @@
         <v>0.6</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>52</v>
       </c>
@@ -2123,7 +2145,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>91</v>
       </c>
@@ -2137,7 +2159,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>92</v>
       </c>
@@ -2154,7 +2176,7 @@
         <v>3.5000000000000003E-2</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>93</v>
       </c>
@@ -2171,7 +2193,7 @@
         <v>8.3999999999999995E-3</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>94</v>
       </c>
@@ -2188,7 +2210,7 @@
         <v>8.4000000000000003E-4</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>95</v>
       </c>
@@ -2202,7 +2224,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>96</v>
       </c>
@@ -2216,7 +2238,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>97</v>
       </c>
@@ -2230,7 +2252,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>98</v>
       </c>
@@ -2244,7 +2266,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>99</v>
       </c>
@@ -2258,7 +2280,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>100</v>
       </c>
@@ -2272,7 +2294,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>155</v>
       </c>
@@ -2290,7 +2312,7 @@
         <v>0.76456000000000002</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>106</v>
       </c>
@@ -2304,7 +2326,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>107</v>
       </c>
@@ -2317,11 +2339,18 @@
       <c r="D77">
         <v>0</v>
       </c>
-      <c r="E77">
+      <c r="E77" s="5">
+        <f>F77/(1-E$52)</f>
+        <v>0.19688004303388917</v>
+      </c>
+      <c r="F77" s="5">
         <v>0.183</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G77" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>108</v>
       </c>
@@ -2334,11 +2363,19 @@
       <c r="D78">
         <v>0</v>
       </c>
-      <c r="E78">
+      <c r="E78" s="5">
+        <f>F78/(1-E$52)</f>
+        <v>0.15169445938676707</v>
+      </c>
+      <c r="F78" s="5">
         <v>0.14099999999999999</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="G78" s="5">
+        <f>F78*F25-E78*E24</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>109</v>
       </c>
@@ -2352,7 +2389,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>110</v>
       </c>
@@ -2436,8 +2473,8 @@
         <v>0</v>
       </c>
       <c r="E85">
-        <f>1-E77-E78-E52</f>
-        <v>0.60549999999999993</v>
+        <f>1-E77-E78</f>
+        <v>0.65142549757934376</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -2667,6 +2704,51 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
+    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </j747ac98061d40f0aa7bd47e1db5675d>
+    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </TaxKeywordTaxHTField>
+    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
+    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
+    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
+    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
+    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Creator>
+    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </EPA_x0020_Contributor>
+    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
+    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </e3f09c3df709400db2417a7161762d62>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -2675,12 +2757,12 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C107526348C97345843FB1F7E3F5FF14" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5efa0b4590ceb4068c523eef838cbf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xmlns:ns3="http://schemas.microsoft.com/sharepoint.v3" xmlns:ns4="http://schemas.microsoft.com/sharepoint/v3/fields" xmlns:ns5="2ba80736-48fa-4d73-aaff-bacaeeed013a" xmlns:ns6="41d9f072-86bf-4c63-b117-debf50ff4701" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9d32b47d5805bf9e4ccfb00021215c68" ns1:_="" ns2:_="" ns3:_="" ns4:_="" ns5:_="" ns6:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -3153,52 +3235,22 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Language xmlns="http://schemas.microsoft.com/sharepoint/v3">English</Language>
-    <j747ac98061d40f0aa7bd47e1db5675d xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </j747ac98061d40f0aa7bd47e1db5675d>
-    <External_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <TaxKeywordTaxHTField xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </TaxKeywordTaxHTField>
-    <Record xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">Shared</Record>
-    <Rights xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <Document_x0020_Creation_x0020_Date xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">2020-10-14T20:30:29+00:00</Document_x0020_Creation_x0020_Date>
-    <EPA_x0020_Office xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <CategoryDescription xmlns="http://schemas.microsoft.com/sharepoint.v3" xsi:nil="true"/>
-    <Identifier xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <_Coverage xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
-    <Creator xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Creator>
-    <EPA_x0020_Related_x0020_Documents xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <EPA_x0020_Contributor xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </EPA_x0020_Contributor>
-    <TaxCatchAll xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4" xsi:nil="true"/>
-    <e3f09c3df709400db2417a7161762d62 xmlns="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </e3f09c3df709400db2417a7161762d62>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="2ba80736-48fa-4d73-aaff-bacaeeed013a">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4DC26B68-A11F-428F-9051-23DC6334A810}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
@@ -3206,7 +3258,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
@@ -3214,7 +3266,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76DF7049-5D71-4C8A-9827-79FC4B574086}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3235,19 +3287,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Highlighted cells where (previous commit) changes were made.
</commit_message>
<xml_diff>
--- a/Inputs/PFOA_template_parameters_Model.xlsx
+++ b/Inputs/PFOA_template_parameters_Model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usepa-my.sharepoint.com/personal/schlosser_paul_epa_gov/Documents/mcsim-5.6.5/PBPK_Model_Template_Mod/Inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="113" documentId="13_ncr:1_{C7746A5F-920D-41F0-A536-A594C5CF14B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{89DA856E-E59D-4561-8B3E-D8CC408A3D95}"/>
+  <xr:revisionPtr revIDLastSave="114" documentId="13_ncr:1_{C7746A5F-920D-41F0-A536-A594C5CF14B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39D21358-F334-452A-BB4D-2533D9DDD551}"/>
   <bookViews>
-    <workbookView xWindow="1830" yWindow="1890" windowWidth="21600" windowHeight="12585" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
+    <workbookView xWindow="-20820" yWindow="840" windowWidth="21600" windowHeight="12585" xr2:uid="{089E7848-11EB-427A-89EA-83825F220BA0}"/>
   </bookViews>
   <sheets>
     <sheet name="MaleRat" sheetId="9" r:id="rId1"/>
@@ -2472,7 +2472,7 @@
       <c r="D85">
         <v>0</v>
       </c>
-      <c r="E85">
+      <c r="E85" s="5">
         <f>1-E77-E78</f>
         <v>0.65142549757934376</v>
       </c>
@@ -2704,6 +2704,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_Source xmlns="http://schemas.microsoft.com/sharepoint/v3/fields" xsi:nil="true"/>
@@ -2746,20 +2760,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="29f62856-1543-49d4-a736-4569d363f533" ContentTypeId="0x0101" PreviousValue="false"/>
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3236,16 +3236,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
-    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
-    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3259,9 +3252,16 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7C4A2D8C-C5B5-46A0-8FC1-3730CC1A83D7}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AA939294-F21F-45CD-81A6-3A616888DAC5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/fields"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="4ffa91fb-a0ff-4ac5-b2db-65c790d184a4"/>
+    <ds:schemaRef ds:uri="93237db7-bebb-43bb-9414-bc3313990c09"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint.v3"/>
+    <ds:schemaRef ds:uri="2ba80736-48fa-4d73-aaff-bacaeeed013a"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>